<commit_message>
Changed Isavia to Avians
</commit_message>
<xml_diff>
--- a/stakeholder_lists.xlsx
+++ b/stakeholder_lists.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\oaolive\repos\mobile-app\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{607F7AEC-318F-4D1B-BBA7-187491980C98}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BDB80D46-EB69-45F5-8786-AC12154E71E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="19440" windowHeight="10320" activeTab="1" xr2:uid="{17D0CF8C-6239-4396-93EE-ED3916C7EA4B}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{17D0CF8C-6239-4396-93EE-ED3916C7EA4B}"/>
   </bookViews>
   <sheets>
     <sheet name="state_lists" sheetId="1" r:id="rId1"/>
@@ -1408,9 +1408,6 @@
     <t>IS_ANSP</t>
   </si>
   <si>
-    <t>Isavia</t>
-  </si>
-  <si>
     <t>IL_ANSP</t>
   </si>
   <si>
@@ -1535,6 +1532,9 @@
   </si>
   <si>
     <t>MUAC_ANSP</t>
+  </si>
+  <si>
+    <t>Avians</t>
   </si>
 </sst>
 </file>
@@ -5370,7 +5370,7 @@
         <v>416</v>
       </c>
       <c r="C1" t="s">
-        <v>497</v>
+        <v>496</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
@@ -5587,7 +5587,7 @@
         <v>455</v>
       </c>
       <c r="B21" t="s">
-        <v>456</v>
+        <v>498</v>
       </c>
       <c r="C21">
         <v>46</v>
@@ -5595,10 +5595,10 @@
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
+        <v>456</v>
+      </c>
+      <c r="B22" t="s">
         <v>457</v>
-      </c>
-      <c r="B22" t="s">
-        <v>458</v>
       </c>
       <c r="C22">
         <v>57</v>
@@ -5606,10 +5606,10 @@
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
+        <v>458</v>
+      </c>
+      <c r="B23" t="s">
         <v>459</v>
-      </c>
-      <c r="B23" t="s">
-        <v>460</v>
       </c>
       <c r="C23">
         <v>33</v>
@@ -5617,10 +5617,10 @@
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
+        <v>460</v>
+      </c>
+      <c r="B24" t="s">
         <v>461</v>
-      </c>
-      <c r="B24" t="s">
-        <v>462</v>
       </c>
       <c r="C24">
         <v>18</v>
@@ -5628,10 +5628,10 @@
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
+        <v>462</v>
+      </c>
+      <c r="B25" t="s">
         <v>463</v>
-      </c>
-      <c r="B25" t="s">
-        <v>464</v>
       </c>
       <c r="C25">
         <v>19</v>
@@ -5639,10 +5639,10 @@
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
+        <v>464</v>
+      </c>
+      <c r="B26" t="s">
         <v>465</v>
-      </c>
-      <c r="B26" t="s">
-        <v>466</v>
       </c>
       <c r="C26">
         <v>20</v>
@@ -5650,10 +5650,10 @@
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
+        <v>466</v>
+      </c>
+      <c r="B27" t="s">
         <v>467</v>
-      </c>
-      <c r="B27" t="s">
-        <v>468</v>
       </c>
       <c r="C27">
         <v>21</v>
@@ -5661,10 +5661,10 @@
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
+        <v>468</v>
+      </c>
+      <c r="B28" t="s">
         <v>469</v>
-      </c>
-      <c r="B28" t="s">
-        <v>470</v>
       </c>
       <c r="C28">
         <v>14</v>
@@ -5672,10 +5672,10 @@
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
+        <v>470</v>
+      </c>
+      <c r="B29" t="s">
         <v>471</v>
-      </c>
-      <c r="B29" t="s">
-        <v>472</v>
       </c>
       <c r="C29">
         <v>22</v>
@@ -5683,7 +5683,7 @@
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>498</v>
+        <v>497</v>
       </c>
       <c r="B30" t="s">
         <v>111</v>
@@ -5694,10 +5694,10 @@
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
+        <v>472</v>
+      </c>
+      <c r="B31" t="s">
         <v>473</v>
-      </c>
-      <c r="B31" t="s">
-        <v>474</v>
       </c>
       <c r="C31">
         <v>26</v>
@@ -5705,10 +5705,10 @@
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
+        <v>474</v>
+      </c>
+      <c r="B32" t="s">
         <v>475</v>
-      </c>
-      <c r="B32" t="s">
-        <v>476</v>
       </c>
       <c r="C32">
         <v>27</v>
@@ -5716,10 +5716,10 @@
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
+        <v>476</v>
+      </c>
+      <c r="B33" t="s">
         <v>477</v>
-      </c>
-      <c r="B33" t="s">
-        <v>478</v>
       </c>
       <c r="C33">
         <v>28</v>
@@ -5727,10 +5727,10 @@
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
+        <v>478</v>
+      </c>
+      <c r="B34" t="s">
         <v>479</v>
-      </c>
-      <c r="B34" t="s">
-        <v>480</v>
       </c>
       <c r="C34">
         <v>56</v>
@@ -5738,10 +5738,10 @@
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
+        <v>480</v>
+      </c>
+      <c r="B35" t="s">
         <v>481</v>
-      </c>
-      <c r="B35" t="s">
-        <v>482</v>
       </c>
       <c r="C35">
         <v>29</v>
@@ -5749,10 +5749,10 @@
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
+        <v>482</v>
+      </c>
+      <c r="B36" t="s">
         <v>483</v>
-      </c>
-      <c r="B36" t="s">
-        <v>484</v>
       </c>
       <c r="C36">
         <v>39</v>
@@ -5760,10 +5760,10 @@
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
+        <v>484</v>
+      </c>
+      <c r="B37" t="s">
         <v>485</v>
-      </c>
-      <c r="B37" t="s">
-        <v>486</v>
       </c>
       <c r="C37">
         <v>30</v>
@@ -5771,10 +5771,10 @@
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
+        <v>486</v>
+      </c>
+      <c r="B38" t="s">
         <v>487</v>
-      </c>
-      <c r="B38" t="s">
-        <v>488</v>
       </c>
       <c r="C38">
         <v>53</v>
@@ -5782,10 +5782,10 @@
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
+        <v>488</v>
+      </c>
+      <c r="B39" t="s">
         <v>489</v>
-      </c>
-      <c r="B39" t="s">
-        <v>490</v>
       </c>
       <c r="C39">
         <v>5</v>
@@ -5793,10 +5793,10 @@
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
+        <v>490</v>
+      </c>
+      <c r="B40" t="s">
         <v>491</v>
-      </c>
-      <c r="B40" t="s">
-        <v>492</v>
       </c>
       <c r="C40">
         <v>31</v>
@@ -5804,10 +5804,10 @@
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
+        <v>492</v>
+      </c>
+      <c r="B41" t="s">
         <v>493</v>
-      </c>
-      <c r="B41" t="s">
-        <v>494</v>
       </c>
       <c r="C41">
         <v>32</v>
@@ -5815,10 +5815,10 @@
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
+        <v>494</v>
+      </c>
+      <c r="B42" t="s">
         <v>495</v>
-      </c>
-      <c r="B42" t="s">
-        <v>496</v>
       </c>
       <c r="C42">
         <v>42</v>

</xml_diff>

<commit_message>
added Marseille TMA to list. created view for acc list and redirected queries to it
</commit_message>
<xml_diff>
--- a/stakeholder_lists.xlsx
+++ b/stakeholder_lists.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\oaolive\repos\mobile-app\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BDB80D46-EB69-45F5-8786-AC12154E71E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D99E359A-C7D7-46A2-801A-FF0E7E0CFD77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{17D0CF8C-6239-4396-93EE-ED3916C7EA4B}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="19440" windowHeight="11520" activeTab="1" xr2:uid="{17D0CF8C-6239-4396-93EE-ED3916C7EA4B}"/>
   </bookViews>
   <sheets>
     <sheet name="state_lists" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1009" uniqueCount="499">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1013" uniqueCount="502">
   <si>
     <t>state</t>
   </si>
@@ -1535,6 +1535,15 @@
   </si>
   <si>
     <t>Avians</t>
+  </si>
+  <si>
+    <t>MARSEILLE APP</t>
+  </si>
+  <si>
+    <t>Marseille TMA</t>
+  </si>
+  <si>
+    <t>LFMMAPP</t>
   </si>
 </sst>
 </file>
@@ -1790,10 +1799,10 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{3B0B9735-26C8-4572-A44C-72BC473CAB08}" name="Table_ACC_NAMES" displayName="Table_ACC_NAMES" ref="A1:D74" totalsRowShown="0">
-  <autoFilter ref="A1:D74" xr:uid="{3B0B9735-26C8-4572-A44C-72BC473CAB08}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:B74">
-    <sortCondition ref="A3:A75"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{3B0B9735-26C8-4572-A44C-72BC473CAB08}" name="Table_ACC_NAMES" displayName="Table_ACC_NAMES" ref="A1:D75" totalsRowShown="0">
+  <autoFilter ref="A1:D75" xr:uid="{3B0B9735-26C8-4572-A44C-72BC473CAB08}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:B75">
+    <sortCondition ref="A3:A76"/>
   </sortState>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{D0688728-A473-461B-9D59-1C5B0693D0A3}" name="NM_name" dataDxfId="3"/>
@@ -4299,7 +4308,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1AE1B1DA-244C-4D7E-AA08-285D46CCB17C}">
-  <dimension ref="A1:D74"/>
+  <dimension ref="A1:D75"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14.7109375" bestFit="1" customWidth="1"/>
@@ -4884,463 +4893,477 @@
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A42" s="5" t="s">
-        <v>316</v>
+        <v>499</v>
       </c>
       <c r="B42" t="s">
-        <v>317</v>
+        <v>500</v>
       </c>
       <c r="C42" t="s">
-        <v>96</v>
+        <v>63</v>
       </c>
       <c r="D42" t="s">
-        <v>318</v>
+        <v>501</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A43" s="5" t="s">
-        <v>319</v>
+        <v>316</v>
       </c>
       <c r="B43" t="s">
-        <v>320</v>
+        <v>317</v>
       </c>
       <c r="C43" t="s">
-        <v>71</v>
+        <v>96</v>
       </c>
       <c r="D43" t="s">
-        <v>321</v>
+        <v>318</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A44" s="5" t="s">
-        <v>322</v>
+        <v>319</v>
       </c>
       <c r="B44" t="s">
-        <v>323</v>
+        <v>320</v>
       </c>
       <c r="C44" t="s">
-        <v>42</v>
+        <v>71</v>
       </c>
       <c r="D44" t="s">
-        <v>324</v>
+        <v>321</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A45" s="5" t="s">
-        <v>325</v>
+        <v>322</v>
       </c>
       <c r="B45" t="s">
-        <v>326</v>
+        <v>323</v>
       </c>
       <c r="C45" t="s">
-        <v>194</v>
+        <v>42</v>
       </c>
       <c r="D45" t="s">
-        <v>327</v>
+        <v>324</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A46" s="5" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
       <c r="B46" t="s">
-        <v>329</v>
+        <v>326</v>
       </c>
       <c r="C46" t="s">
-        <v>136</v>
+        <v>194</v>
       </c>
       <c r="D46" t="s">
-        <v>330</v>
+        <v>327</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A47" s="5" t="s">
-        <v>331</v>
+        <v>328</v>
       </c>
       <c r="B47" t="s">
-        <v>332</v>
+        <v>329</v>
       </c>
       <c r="C47" t="s">
-        <v>96</v>
+        <v>136</v>
       </c>
       <c r="D47" t="s">
-        <v>333</v>
+        <v>330</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A48" s="5" t="s">
-        <v>334</v>
+        <v>331</v>
       </c>
       <c r="B48" t="s">
-        <v>335</v>
+        <v>332</v>
       </c>
       <c r="C48" t="s">
-        <v>167</v>
+        <v>96</v>
       </c>
       <c r="D48" t="s">
-        <v>336</v>
+        <v>333</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A49" s="5" t="s">
-        <v>337</v>
+        <v>334</v>
       </c>
       <c r="B49" t="s">
-        <v>338</v>
+        <v>335</v>
       </c>
       <c r="C49" t="s">
-        <v>63</v>
+        <v>167</v>
       </c>
       <c r="D49" t="s">
-        <v>339</v>
+        <v>336</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A50" s="5" t="s">
-        <v>340</v>
+        <v>337</v>
       </c>
       <c r="B50" t="s">
-        <v>341</v>
+        <v>338</v>
       </c>
       <c r="C50" t="s">
-        <v>46</v>
+        <v>63</v>
       </c>
       <c r="D50" t="s">
-        <v>342</v>
+        <v>339</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A51" s="5" t="s">
-        <v>343</v>
+        <v>340</v>
       </c>
       <c r="B51" t="s">
-        <v>344</v>
+        <v>341</v>
       </c>
       <c r="C51" t="s">
-        <v>63</v>
+        <v>46</v>
       </c>
       <c r="D51" t="s">
-        <v>345</v>
+        <v>342</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A52" s="5" t="s">
-        <v>346</v>
+        <v>343</v>
       </c>
       <c r="B52" t="s">
-        <v>347</v>
+        <v>344</v>
       </c>
       <c r="C52" t="s">
-        <v>83</v>
+        <v>63</v>
       </c>
       <c r="D52" t="s">
-        <v>348</v>
+        <v>345</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A53" s="5" t="s">
-        <v>349</v>
+        <v>346</v>
       </c>
       <c r="B53" t="s">
-        <v>350</v>
+        <v>347</v>
       </c>
       <c r="C53" t="s">
-        <v>100</v>
+        <v>83</v>
       </c>
       <c r="D53" t="s">
-        <v>351</v>
+        <v>348</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A54" s="5" t="s">
-        <v>352</v>
+        <v>349</v>
       </c>
       <c r="B54" t="s">
-        <v>353</v>
+        <v>350</v>
       </c>
       <c r="C54" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="D54" t="s">
-        <v>354</v>
+        <v>351</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A55" s="5" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
       <c r="B55" t="s">
-        <v>356</v>
+        <v>353</v>
       </c>
       <c r="C55" t="s">
-        <v>146</v>
+        <v>96</v>
       </c>
       <c r="D55" t="s">
-        <v>357</v>
+        <v>354</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A56" s="5" t="s">
-        <v>358</v>
+        <v>355</v>
       </c>
       <c r="B56" t="s">
-        <v>359</v>
+        <v>356</v>
       </c>
       <c r="C56" t="s">
-        <v>28</v>
+        <v>146</v>
       </c>
       <c r="D56" t="s">
-        <v>360</v>
+        <v>357</v>
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A57" s="5" t="s">
-        <v>361</v>
+        <v>358</v>
       </c>
       <c r="B57" t="s">
-        <v>362</v>
+        <v>359</v>
       </c>
       <c r="C57" t="s">
-        <v>188</v>
+        <v>28</v>
       </c>
       <c r="D57" t="s">
-        <v>363</v>
+        <v>360</v>
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A58" s="5" t="s">
-        <v>364</v>
+        <v>361</v>
       </c>
       <c r="B58" t="s">
-        <v>365</v>
+        <v>362</v>
       </c>
       <c r="C58" t="s">
-        <v>167</v>
+        <v>188</v>
       </c>
       <c r="D58" t="s">
-        <v>366</v>
+        <v>363</v>
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A59" s="5" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="B59" t="s">
-        <v>368</v>
+        <v>365</v>
       </c>
       <c r="C59" t="s">
-        <v>88</v>
+        <v>167</v>
       </c>
       <c r="D59" t="s">
-        <v>369</v>
+        <v>366</v>
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A60" s="5" t="s">
-        <v>370</v>
+        <v>367</v>
       </c>
       <c r="B60" t="s">
-        <v>371</v>
+        <v>368</v>
       </c>
       <c r="C60" t="s">
-        <v>188</v>
+        <v>88</v>
       </c>
       <c r="D60" t="s">
-        <v>372</v>
+        <v>369</v>
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A61" s="5" t="s">
-        <v>373</v>
+        <v>370</v>
       </c>
       <c r="B61" t="s">
-        <v>374</v>
+        <v>371</v>
       </c>
       <c r="C61" t="s">
-        <v>132</v>
+        <v>188</v>
       </c>
       <c r="D61" t="s">
-        <v>375</v>
+        <v>372</v>
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A62" s="5" t="s">
-        <v>376</v>
+        <v>373</v>
       </c>
       <c r="B62" t="s">
-        <v>377</v>
+        <v>374</v>
       </c>
       <c r="C62" t="s">
-        <v>32</v>
+        <v>132</v>
       </c>
       <c r="D62" t="s">
-        <v>378</v>
+        <v>375</v>
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A63" s="5" t="s">
-        <v>379</v>
+        <v>376</v>
       </c>
       <c r="B63" t="s">
-        <v>380</v>
+        <v>377</v>
       </c>
       <c r="C63" t="s">
-        <v>136</v>
+        <v>32</v>
       </c>
       <c r="D63" t="s">
-        <v>381</v>
+        <v>378</v>
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A64" s="5" t="s">
-        <v>382</v>
+        <v>379</v>
       </c>
       <c r="B64" t="s">
-        <v>383</v>
+        <v>380</v>
       </c>
       <c r="C64" t="s">
-        <v>171</v>
+        <v>136</v>
       </c>
       <c r="D64" t="s">
-        <v>384</v>
+        <v>381</v>
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A65" s="5" t="s">
-        <v>385</v>
+        <v>382</v>
       </c>
       <c r="B65" t="s">
-        <v>386</v>
+        <v>383</v>
       </c>
       <c r="C65" t="s">
-        <v>55</v>
+        <v>171</v>
       </c>
       <c r="D65" t="s">
-        <v>387</v>
+        <v>384</v>
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A66" s="5" t="s">
-        <v>388</v>
+        <v>385</v>
       </c>
       <c r="B66" t="s">
-        <v>389</v>
+        <v>386</v>
       </c>
       <c r="C66" t="s">
-        <v>67</v>
+        <v>55</v>
       </c>
       <c r="D66" t="s">
-        <v>390</v>
+        <v>387</v>
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A67" s="5" t="s">
-        <v>391</v>
+        <v>388</v>
       </c>
       <c r="B67" t="s">
-        <v>392</v>
+        <v>389</v>
       </c>
       <c r="C67" t="s">
-        <v>93</v>
+        <v>67</v>
       </c>
       <c r="D67" t="s">
-        <v>393</v>
+        <v>390</v>
       </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A68" s="5" t="s">
-        <v>394</v>
+        <v>391</v>
       </c>
       <c r="B68" t="s">
-        <v>395</v>
+        <v>392</v>
       </c>
       <c r="C68" t="s">
-        <v>10</v>
+        <v>93</v>
       </c>
       <c r="D68" t="s">
-        <v>396</v>
+        <v>393</v>
       </c>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A69" s="5" t="s">
-        <v>397</v>
+        <v>394</v>
       </c>
       <c r="B69" t="s">
-        <v>398</v>
+        <v>395</v>
       </c>
       <c r="C69" t="s">
-        <v>104</v>
+        <v>10</v>
       </c>
       <c r="D69" t="s">
-        <v>399</v>
+        <v>396</v>
       </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A70" s="5" t="s">
-        <v>400</v>
+        <v>397</v>
       </c>
       <c r="B70" t="s">
-        <v>401</v>
+        <v>398</v>
       </c>
       <c r="C70" t="s">
-        <v>140</v>
+        <v>104</v>
       </c>
       <c r="D70" t="s">
-        <v>402</v>
+        <v>399</v>
       </c>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A71" s="5" t="s">
-        <v>403</v>
+        <v>400</v>
       </c>
       <c r="B71" t="s">
-        <v>404</v>
+        <v>401</v>
       </c>
       <c r="C71" t="s">
-        <v>18</v>
+        <v>140</v>
       </c>
       <c r="D71" t="s">
-        <v>405</v>
+        <v>402</v>
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A72" s="5" t="s">
-        <v>406</v>
+        <v>403</v>
       </c>
       <c r="B72" t="s">
-        <v>407</v>
+        <v>404</v>
       </c>
       <c r="C72" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="D72" t="s">
-        <v>408</v>
+        <v>405</v>
       </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A73" s="5" t="s">
+        <v>406</v>
+      </c>
+      <c r="B73" t="s">
+        <v>407</v>
+      </c>
+      <c r="C73" t="s">
+        <v>14</v>
+      </c>
+      <c r="D73" t="s">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="74" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A74" s="5" t="s">
         <v>409</v>
       </c>
-      <c r="B73" t="s">
+      <c r="B74" t="s">
         <v>410</v>
       </c>
-      <c r="C73" t="s">
+      <c r="C74" t="s">
         <v>36</v>
       </c>
-      <c r="D73" t="s">
+      <c r="D74" t="s">
         <v>411</v>
       </c>
     </row>
-    <row r="74" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A74" s="6" t="s">
+    <row r="75" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A75" s="6" t="s">
         <v>412</v>
       </c>
-      <c r="B74" t="s">
+      <c r="B75" t="s">
         <v>413</v>
       </c>
-      <c r="C74" t="s">
+      <c r="C75" t="s">
         <v>179</v>
       </c>
-      <c r="D74" t="s">
+      <c r="D75" t="s">
         <v>414</v>
       </c>
     </row>

</xml_diff>

<commit_message>
added marseille exception to acc map code
</commit_message>
<xml_diff>
--- a/stakeholder_lists.xlsx
+++ b/stakeholder_lists.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\oaolive\repos\mobile-app\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D99E359A-C7D7-46A2-801A-FF0E7E0CFD77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8FAAE808-5D50-4EBB-B7F7-03082F7D7B6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="19440" windowHeight="11520" activeTab="1" xr2:uid="{17D0CF8C-6239-4396-93EE-ED3916C7EA4B}"/>
   </bookViews>
@@ -919,9 +919,6 @@
     <t>LONDON TMA TC</t>
   </si>
   <si>
-    <t>London TMA TC</t>
-  </si>
-  <si>
     <t>EGTTTC</t>
   </si>
   <si>
@@ -1544,6 +1541,9 @@
   </si>
   <si>
     <t>LFMMAPP</t>
+  </si>
+  <si>
+    <t>London TMA</t>
   </si>
 </sst>
 </file>
@@ -4784,587 +4784,587 @@
         <v>292</v>
       </c>
       <c r="B34" t="s">
-        <v>293</v>
+        <v>501</v>
       </c>
       <c r="C34" t="s">
         <v>188</v>
       </c>
       <c r="D34" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A35" s="5" t="s">
+        <v>294</v>
+      </c>
+      <c r="B35" t="s">
         <v>295</v>
-      </c>
-      <c r="B35" t="s">
-        <v>296</v>
       </c>
       <c r="C35" t="s">
         <v>194</v>
       </c>
       <c r="D35" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A36" s="5" t="s">
+        <v>297</v>
+      </c>
+      <c r="B36" t="s">
         <v>298</v>
-      </c>
-      <c r="B36" t="s">
-        <v>299</v>
       </c>
       <c r="C36" t="s">
         <v>111</v>
       </c>
       <c r="D36" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A37" s="5" t="s">
+        <v>300</v>
+      </c>
+      <c r="B37" t="s">
         <v>301</v>
-      </c>
-      <c r="B37" t="s">
-        <v>302</v>
       </c>
       <c r="C37" t="s">
         <v>167</v>
       </c>
       <c r="D37" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A38" s="5" t="s">
+        <v>303</v>
+      </c>
+      <c r="B38" t="s">
         <v>304</v>
-      </c>
-      <c r="B38" t="s">
-        <v>305</v>
       </c>
       <c r="C38" t="s">
         <v>75</v>
       </c>
       <c r="D38" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A39" s="5" t="s">
+        <v>306</v>
+      </c>
+      <c r="B39" t="s">
         <v>307</v>
-      </c>
-      <c r="B39" t="s">
-        <v>308</v>
       </c>
       <c r="C39" t="s">
         <v>171</v>
       </c>
       <c r="D39" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A40" s="5" t="s">
+        <v>309</v>
+      </c>
+      <c r="B40" t="s">
         <v>310</v>
-      </c>
-      <c r="B40" t="s">
-        <v>311</v>
       </c>
       <c r="C40" t="s">
         <v>113</v>
       </c>
       <c r="D40" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A41" s="5" t="s">
+        <v>312</v>
+      </c>
+      <c r="B41" t="s">
         <v>313</v>
-      </c>
-      <c r="B41" t="s">
-        <v>314</v>
       </c>
       <c r="C41" t="s">
         <v>63</v>
       </c>
       <c r="D41" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A42" s="5" t="s">
+        <v>498</v>
+      </c>
+      <c r="B42" t="s">
         <v>499</v>
-      </c>
-      <c r="B42" t="s">
-        <v>500</v>
       </c>
       <c r="C42" t="s">
         <v>63</v>
       </c>
       <c r="D42" t="s">
-        <v>501</v>
+        <v>500</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A43" s="5" t="s">
+        <v>315</v>
+      </c>
+      <c r="B43" t="s">
         <v>316</v>
-      </c>
-      <c r="B43" t="s">
-        <v>317</v>
       </c>
       <c r="C43" t="s">
         <v>96</v>
       </c>
       <c r="D43" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A44" s="5" t="s">
+        <v>318</v>
+      </c>
+      <c r="B44" t="s">
         <v>319</v>
-      </c>
-      <c r="B44" t="s">
-        <v>320</v>
       </c>
       <c r="C44" t="s">
         <v>71</v>
       </c>
       <c r="D44" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A45" s="5" t="s">
+        <v>321</v>
+      </c>
+      <c r="B45" t="s">
         <v>322</v>
-      </c>
-      <c r="B45" t="s">
-        <v>323</v>
       </c>
       <c r="C45" t="s">
         <v>42</v>
       </c>
       <c r="D45" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A46" s="5" t="s">
+        <v>324</v>
+      </c>
+      <c r="B46" t="s">
         <v>325</v>
-      </c>
-      <c r="B46" t="s">
-        <v>326</v>
       </c>
       <c r="C46" t="s">
         <v>194</v>
       </c>
       <c r="D46" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A47" s="5" t="s">
+        <v>327</v>
+      </c>
+      <c r="B47" t="s">
         <v>328</v>
-      </c>
-      <c r="B47" t="s">
-        <v>329</v>
       </c>
       <c r="C47" t="s">
         <v>136</v>
       </c>
       <c r="D47" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A48" s="5" t="s">
+        <v>330</v>
+      </c>
+      <c r="B48" t="s">
         <v>331</v>
-      </c>
-      <c r="B48" t="s">
-        <v>332</v>
       </c>
       <c r="C48" t="s">
         <v>96</v>
       </c>
       <c r="D48" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A49" s="5" t="s">
+        <v>333</v>
+      </c>
+      <c r="B49" t="s">
         <v>334</v>
-      </c>
-      <c r="B49" t="s">
-        <v>335</v>
       </c>
       <c r="C49" t="s">
         <v>167</v>
       </c>
       <c r="D49" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A50" s="5" t="s">
+        <v>336</v>
+      </c>
+      <c r="B50" t="s">
         <v>337</v>
-      </c>
-      <c r="B50" t="s">
-        <v>338</v>
       </c>
       <c r="C50" t="s">
         <v>63</v>
       </c>
       <c r="D50" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A51" s="5" t="s">
+        <v>339</v>
+      </c>
+      <c r="B51" t="s">
         <v>340</v>
-      </c>
-      <c r="B51" t="s">
-        <v>341</v>
       </c>
       <c r="C51" t="s">
         <v>46</v>
       </c>
       <c r="D51" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A52" s="5" t="s">
+        <v>342</v>
+      </c>
+      <c r="B52" t="s">
         <v>343</v>
-      </c>
-      <c r="B52" t="s">
-        <v>344</v>
       </c>
       <c r="C52" t="s">
         <v>63</v>
       </c>
       <c r="D52" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A53" s="5" t="s">
+        <v>345</v>
+      </c>
+      <c r="B53" t="s">
         <v>346</v>
-      </c>
-      <c r="B53" t="s">
-        <v>347</v>
       </c>
       <c r="C53" t="s">
         <v>83</v>
       </c>
       <c r="D53" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A54" s="5" t="s">
+        <v>348</v>
+      </c>
+      <c r="B54" t="s">
         <v>349</v>
-      </c>
-      <c r="B54" t="s">
-        <v>350</v>
       </c>
       <c r="C54" t="s">
         <v>100</v>
       </c>
       <c r="D54" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A55" s="5" t="s">
+        <v>351</v>
+      </c>
+      <c r="B55" t="s">
         <v>352</v>
-      </c>
-      <c r="B55" t="s">
-        <v>353</v>
       </c>
       <c r="C55" t="s">
         <v>96</v>
       </c>
       <c r="D55" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A56" s="5" t="s">
+        <v>354</v>
+      </c>
+      <c r="B56" t="s">
         <v>355</v>
-      </c>
-      <c r="B56" t="s">
-        <v>356</v>
       </c>
       <c r="C56" t="s">
         <v>146</v>
       </c>
       <c r="D56" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A57" s="5" t="s">
+        <v>357</v>
+      </c>
+      <c r="B57" t="s">
         <v>358</v>
-      </c>
-      <c r="B57" t="s">
-        <v>359</v>
       </c>
       <c r="C57" t="s">
         <v>28</v>
       </c>
       <c r="D57" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A58" s="5" t="s">
+        <v>360</v>
+      </c>
+      <c r="B58" t="s">
         <v>361</v>
-      </c>
-      <c r="B58" t="s">
-        <v>362</v>
       </c>
       <c r="C58" t="s">
         <v>188</v>
       </c>
       <c r="D58" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A59" s="5" t="s">
+        <v>363</v>
+      </c>
+      <c r="B59" t="s">
         <v>364</v>
-      </c>
-      <c r="B59" t="s">
-        <v>365</v>
       </c>
       <c r="C59" t="s">
         <v>167</v>
       </c>
       <c r="D59" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A60" s="5" t="s">
+        <v>366</v>
+      </c>
+      <c r="B60" t="s">
         <v>367</v>
-      </c>
-      <c r="B60" t="s">
-        <v>368</v>
       </c>
       <c r="C60" t="s">
         <v>88</v>
       </c>
       <c r="D60" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A61" s="5" t="s">
+        <v>369</v>
+      </c>
+      <c r="B61" t="s">
         <v>370</v>
-      </c>
-      <c r="B61" t="s">
-        <v>371</v>
       </c>
       <c r="C61" t="s">
         <v>188</v>
       </c>
       <c r="D61" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A62" s="5" t="s">
+        <v>372</v>
+      </c>
+      <c r="B62" t="s">
         <v>373</v>
-      </c>
-      <c r="B62" t="s">
-        <v>374</v>
       </c>
       <c r="C62" t="s">
         <v>132</v>
       </c>
       <c r="D62" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A63" s="5" t="s">
+        <v>375</v>
+      </c>
+      <c r="B63" t="s">
         <v>376</v>
-      </c>
-      <c r="B63" t="s">
-        <v>377</v>
       </c>
       <c r="C63" t="s">
         <v>32</v>
       </c>
       <c r="D63" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A64" s="5" t="s">
+        <v>378</v>
+      </c>
+      <c r="B64" t="s">
         <v>379</v>
-      </c>
-      <c r="B64" t="s">
-        <v>380</v>
       </c>
       <c r="C64" t="s">
         <v>136</v>
       </c>
       <c r="D64" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A65" s="5" t="s">
+        <v>381</v>
+      </c>
+      <c r="B65" t="s">
         <v>382</v>
-      </c>
-      <c r="B65" t="s">
-        <v>383</v>
       </c>
       <c r="C65" t="s">
         <v>171</v>
       </c>
       <c r="D65" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A66" s="5" t="s">
+        <v>384</v>
+      </c>
+      <c r="B66" t="s">
         <v>385</v>
-      </c>
-      <c r="B66" t="s">
-        <v>386</v>
       </c>
       <c r="C66" t="s">
         <v>55</v>
       </c>
       <c r="D66" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A67" s="5" t="s">
+        <v>387</v>
+      </c>
+      <c r="B67" t="s">
         <v>388</v>
-      </c>
-      <c r="B67" t="s">
-        <v>389</v>
       </c>
       <c r="C67" t="s">
         <v>67</v>
       </c>
       <c r="D67" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A68" s="5" t="s">
+        <v>390</v>
+      </c>
+      <c r="B68" t="s">
         <v>391</v>
-      </c>
-      <c r="B68" t="s">
-        <v>392</v>
       </c>
       <c r="C68" t="s">
         <v>93</v>
       </c>
       <c r="D68" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A69" s="5" t="s">
+        <v>393</v>
+      </c>
+      <c r="B69" t="s">
         <v>394</v>
-      </c>
-      <c r="B69" t="s">
-        <v>395</v>
       </c>
       <c r="C69" t="s">
         <v>10</v>
       </c>
       <c r="D69" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A70" s="5" t="s">
+        <v>396</v>
+      </c>
+      <c r="B70" t="s">
         <v>397</v>
-      </c>
-      <c r="B70" t="s">
-        <v>398</v>
       </c>
       <c r="C70" t="s">
         <v>104</v>
       </c>
       <c r="D70" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A71" s="5" t="s">
+        <v>399</v>
+      </c>
+      <c r="B71" t="s">
         <v>400</v>
-      </c>
-      <c r="B71" t="s">
-        <v>401</v>
       </c>
       <c r="C71" t="s">
         <v>140</v>
       </c>
       <c r="D71" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A72" s="5" t="s">
+        <v>402</v>
+      </c>
+      <c r="B72" t="s">
         <v>403</v>
-      </c>
-      <c r="B72" t="s">
-        <v>404</v>
       </c>
       <c r="C72" t="s">
         <v>18</v>
       </c>
       <c r="D72" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A73" s="5" t="s">
+        <v>405</v>
+      </c>
+      <c r="B73" t="s">
         <v>406</v>
-      </c>
-      <c r="B73" t="s">
-        <v>407</v>
       </c>
       <c r="C73" t="s">
         <v>14</v>
       </c>
       <c r="D73" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A74" s="5" t="s">
+        <v>408</v>
+      </c>
+      <c r="B74" t="s">
         <v>409</v>
-      </c>
-      <c r="B74" t="s">
-        <v>410</v>
       </c>
       <c r="C74" t="s">
         <v>36</v>
       </c>
       <c r="D74" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A75" s="6" t="s">
+        <v>411</v>
+      </c>
+      <c r="B75" t="s">
         <v>412</v>
-      </c>
-      <c r="B75" t="s">
-        <v>413</v>
       </c>
       <c r="C75" t="s">
         <v>179</v>
       </c>
       <c r="D75" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
     </row>
   </sheetData>
@@ -5387,21 +5387,21 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>414</v>
+      </c>
+      <c r="B1" t="s">
         <v>415</v>
       </c>
-      <c r="B1" t="s">
-        <v>416</v>
-      </c>
       <c r="C1" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>416</v>
+      </c>
+      <c r="B2" t="s">
         <v>417</v>
-      </c>
-      <c r="B2" t="s">
-        <v>418</v>
       </c>
       <c r="C2">
         <v>17</v>
@@ -5409,10 +5409,10 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>418</v>
+      </c>
+      <c r="B3" t="s">
         <v>419</v>
-      </c>
-      <c r="B3" t="s">
-        <v>420</v>
       </c>
       <c r="C3">
         <v>24</v>
@@ -5420,10 +5420,10 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>420</v>
+      </c>
+      <c r="B4" t="s">
         <v>421</v>
-      </c>
-      <c r="B4" t="s">
-        <v>422</v>
       </c>
       <c r="C4">
         <v>2</v>
@@ -5431,10 +5431,10 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>422</v>
+      </c>
+      <c r="B5" t="s">
         <v>423</v>
-      </c>
-      <c r="B5" t="s">
-        <v>424</v>
       </c>
       <c r="C5">
         <v>44</v>
@@ -5442,10 +5442,10 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>424</v>
+      </c>
+      <c r="B6" t="s">
         <v>425</v>
-      </c>
-      <c r="B6" t="s">
-        <v>426</v>
       </c>
       <c r="C6">
         <v>4</v>
@@ -5453,10 +5453,10 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>426</v>
+      </c>
+      <c r="B7" t="s">
         <v>427</v>
-      </c>
-      <c r="B7" t="s">
-        <v>428</v>
       </c>
       <c r="C7">
         <v>50</v>
@@ -5464,10 +5464,10 @@
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
+        <v>428</v>
+      </c>
+      <c r="B8" t="s">
         <v>429</v>
-      </c>
-      <c r="B8" t="s">
-        <v>430</v>
       </c>
       <c r="C8">
         <v>45</v>
@@ -5475,10 +5475,10 @@
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
+        <v>430</v>
+      </c>
+      <c r="B9" t="s">
         <v>431</v>
-      </c>
-      <c r="B9" t="s">
-        <v>432</v>
       </c>
       <c r="C9">
         <v>3</v>
@@ -5486,10 +5486,10 @@
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
+        <v>432</v>
+      </c>
+      <c r="B10" t="s">
         <v>433</v>
-      </c>
-      <c r="B10" t="s">
-        <v>434</v>
       </c>
       <c r="C10">
         <v>6</v>
@@ -5497,10 +5497,10 @@
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
+        <v>434</v>
+      </c>
+      <c r="B11" t="s">
         <v>435</v>
-      </c>
-      <c r="B11" t="s">
-        <v>436</v>
       </c>
       <c r="C11">
         <v>7</v>
@@ -5508,10 +5508,10 @@
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
+        <v>436</v>
+      </c>
+      <c r="B12" t="s">
         <v>437</v>
-      </c>
-      <c r="B12" t="s">
-        <v>438</v>
       </c>
       <c r="C12">
         <v>8</v>
@@ -5519,10 +5519,10 @@
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
+        <v>438</v>
+      </c>
+      <c r="B13" t="s">
         <v>439</v>
-      </c>
-      <c r="B13" t="s">
-        <v>440</v>
       </c>
       <c r="C13">
         <v>9</v>
@@ -5530,10 +5530,10 @@
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
+        <v>440</v>
+      </c>
+      <c r="B14" t="s">
         <v>441</v>
-      </c>
-      <c r="B14" t="s">
-        <v>442</v>
       </c>
       <c r="C14">
         <v>10</v>
@@ -5541,10 +5541,10 @@
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
+        <v>442</v>
+      </c>
+      <c r="B15" t="s">
         <v>443</v>
-      </c>
-      <c r="B15" t="s">
-        <v>444</v>
       </c>
       <c r="C15">
         <v>11</v>
@@ -5552,10 +5552,10 @@
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
+        <v>444</v>
+      </c>
+      <c r="B16" t="s">
         <v>445</v>
-      </c>
-      <c r="B16" t="s">
-        <v>446</v>
       </c>
       <c r="C16">
         <v>1</v>
@@ -5563,10 +5563,10 @@
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
+        <v>446</v>
+      </c>
+      <c r="B17" t="s">
         <v>447</v>
-      </c>
-      <c r="B17" t="s">
-        <v>448</v>
       </c>
       <c r="C17">
         <v>12</v>
@@ -5574,10 +5574,10 @@
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
+        <v>448</v>
+      </c>
+      <c r="B18" t="s">
         <v>449</v>
-      </c>
-      <c r="B18" t="s">
-        <v>450</v>
       </c>
       <c r="C18">
         <v>13</v>
@@ -5585,10 +5585,10 @@
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
+        <v>450</v>
+      </c>
+      <c r="B19" t="s">
         <v>451</v>
-      </c>
-      <c r="B19" t="s">
-        <v>452</v>
       </c>
       <c r="C19">
         <v>15</v>
@@ -5596,10 +5596,10 @@
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
+        <v>452</v>
+      </c>
+      <c r="B20" t="s">
         <v>453</v>
-      </c>
-      <c r="B20" t="s">
-        <v>454</v>
       </c>
       <c r="C20">
         <v>16</v>
@@ -5607,10 +5607,10 @@
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>455</v>
+        <v>454</v>
       </c>
       <c r="B21" t="s">
-        <v>498</v>
+        <v>497</v>
       </c>
       <c r="C21">
         <v>46</v>
@@ -5618,10 +5618,10 @@
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
+        <v>455</v>
+      </c>
+      <c r="B22" t="s">
         <v>456</v>
-      </c>
-      <c r="B22" t="s">
-        <v>457</v>
       </c>
       <c r="C22">
         <v>57</v>
@@ -5629,10 +5629,10 @@
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
+        <v>457</v>
+      </c>
+      <c r="B23" t="s">
         <v>458</v>
-      </c>
-      <c r="B23" t="s">
-        <v>459</v>
       </c>
       <c r="C23">
         <v>33</v>
@@ -5640,10 +5640,10 @@
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
+        <v>459</v>
+      </c>
+      <c r="B24" t="s">
         <v>460</v>
-      </c>
-      <c r="B24" t="s">
-        <v>461</v>
       </c>
       <c r="C24">
         <v>18</v>
@@ -5651,10 +5651,10 @@
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
+        <v>461</v>
+      </c>
+      <c r="B25" t="s">
         <v>462</v>
-      </c>
-      <c r="B25" t="s">
-        <v>463</v>
       </c>
       <c r="C25">
         <v>19</v>
@@ -5662,10 +5662,10 @@
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
+        <v>463</v>
+      </c>
+      <c r="B26" t="s">
         <v>464</v>
-      </c>
-      <c r="B26" t="s">
-        <v>465</v>
       </c>
       <c r="C26">
         <v>20</v>
@@ -5673,10 +5673,10 @@
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
+        <v>465</v>
+      </c>
+      <c r="B27" t="s">
         <v>466</v>
-      </c>
-      <c r="B27" t="s">
-        <v>467</v>
       </c>
       <c r="C27">
         <v>21</v>
@@ -5684,10 +5684,10 @@
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
+        <v>467</v>
+      </c>
+      <c r="B28" t="s">
         <v>468</v>
-      </c>
-      <c r="B28" t="s">
-        <v>469</v>
       </c>
       <c r="C28">
         <v>14</v>
@@ -5695,10 +5695,10 @@
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
+        <v>469</v>
+      </c>
+      <c r="B29" t="s">
         <v>470</v>
-      </c>
-      <c r="B29" t="s">
-        <v>471</v>
       </c>
       <c r="C29">
         <v>22</v>
@@ -5706,7 +5706,7 @@
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>497</v>
+        <v>496</v>
       </c>
       <c r="B30" t="s">
         <v>111</v>
@@ -5717,10 +5717,10 @@
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
+        <v>471</v>
+      </c>
+      <c r="B31" t="s">
         <v>472</v>
-      </c>
-      <c r="B31" t="s">
-        <v>473</v>
       </c>
       <c r="C31">
         <v>26</v>
@@ -5728,10 +5728,10 @@
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
+        <v>473</v>
+      </c>
+      <c r="B32" t="s">
         <v>474</v>
-      </c>
-      <c r="B32" t="s">
-        <v>475</v>
       </c>
       <c r="C32">
         <v>27</v>
@@ -5739,10 +5739,10 @@
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
+        <v>475</v>
+      </c>
+      <c r="B33" t="s">
         <v>476</v>
-      </c>
-      <c r="B33" t="s">
-        <v>477</v>
       </c>
       <c r="C33">
         <v>28</v>
@@ -5750,10 +5750,10 @@
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
+        <v>477</v>
+      </c>
+      <c r="B34" t="s">
         <v>478</v>
-      </c>
-      <c r="B34" t="s">
-        <v>479</v>
       </c>
       <c r="C34">
         <v>56</v>
@@ -5761,10 +5761,10 @@
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
+        <v>479</v>
+      </c>
+      <c r="B35" t="s">
         <v>480</v>
-      </c>
-      <c r="B35" t="s">
-        <v>481</v>
       </c>
       <c r="C35">
         <v>29</v>
@@ -5772,10 +5772,10 @@
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
+        <v>481</v>
+      </c>
+      <c r="B36" t="s">
         <v>482</v>
-      </c>
-      <c r="B36" t="s">
-        <v>483</v>
       </c>
       <c r="C36">
         <v>39</v>
@@ -5783,10 +5783,10 @@
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
+        <v>483</v>
+      </c>
+      <c r="B37" t="s">
         <v>484</v>
-      </c>
-      <c r="B37" t="s">
-        <v>485</v>
       </c>
       <c r="C37">
         <v>30</v>
@@ -5794,10 +5794,10 @@
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
+        <v>485</v>
+      </c>
+      <c r="B38" t="s">
         <v>486</v>
-      </c>
-      <c r="B38" t="s">
-        <v>487</v>
       </c>
       <c r="C38">
         <v>53</v>
@@ -5805,10 +5805,10 @@
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
+        <v>487</v>
+      </c>
+      <c r="B39" t="s">
         <v>488</v>
-      </c>
-      <c r="B39" t="s">
-        <v>489</v>
       </c>
       <c r="C39">
         <v>5</v>
@@ -5816,10 +5816,10 @@
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
+        <v>489</v>
+      </c>
+      <c r="B40" t="s">
         <v>490</v>
-      </c>
-      <c r="B40" t="s">
-        <v>491</v>
       </c>
       <c r="C40">
         <v>31</v>
@@ -5827,10 +5827,10 @@
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
+        <v>491</v>
+      </c>
+      <c r="B41" t="s">
         <v>492</v>
-      </c>
-      <c r="B41" t="s">
-        <v>493</v>
       </c>
       <c r="C41">
         <v>32</v>
@@ -5838,10 +5838,10 @@
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
+        <v>493</v>
+      </c>
+      <c r="B42" t="s">
         <v>494</v>
-      </c>
-      <c r="B42" t="s">
-        <v>495</v>
       </c>
       <c r="C42">
         <v>42</v>

</xml_diff>